<commit_message>
version 41 - Fix display for admin right
</commit_message>
<xml_diff>
--- a/Documentation/Database_Architecture/Database_design_architecture.xlsx
+++ b/Documentation/Database_Architecture/Database_design_architecture.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="237">
   <si>
     <t>Model for SQL and No SQL combination</t>
   </si>
@@ -770,6 +770,18 @@
   </si>
   <si>
     <t>Read quantity of product based on product name</t>
+  </si>
+  <si>
+    <t>INSERT INTO inventory (product_sku,quantity,warehouse_id) VALUES ('${Product_name}',${Product_quantity},${Product_area});</t>
+  </si>
+  <si>
+    <t>Add new product with quantity and location for admin right</t>
+  </si>
+  <si>
+    <t>DELETE from inventory WHERE product_sku = '${Product_name}'</t>
+  </si>
+  <si>
+    <t>Delete product for admin right</t>
   </si>
   <si>
     <t>Table 7</t>
@@ -3631,7 +3643,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3505200" y="20425410"/>
+          <a:off x="3505200" y="20684490"/>
           <a:ext cx="7581900" cy="5095875"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5108,22 +5120,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="16:16">
       <c r="P4" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="16:16">
       <c r="P6" s="7" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" spans="16:16">
       <c r="P7" s="7" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -5149,17 +5161,17 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="9:9">
       <c r="I11" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13" spans="9:9">
       <c r="I13" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -5182,7 +5194,7 @@
   <sheetData>
     <row r="21" spans="1:1">
       <c r="A21" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -5208,7 +5220,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -5234,7 +5246,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -5260,7 +5272,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -5286,172 +5298,172 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" ht="25.8" spans="2:2">
       <c r="B3" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" ht="21" spans="2:2">
       <c r="B5" s="3" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="3:3">
       <c r="C8" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="3:3">
       <c r="C9" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="3:3">
       <c r="C10" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="3:3">
       <c r="C11" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="3:3">
       <c r="C12" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="3:3">
       <c r="C13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="3:3">
       <c r="C14" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
     </row>
     <row r="15" spans="3:3">
       <c r="C15" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="3:3">
       <c r="C16" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="19" ht="21" spans="2:2">
       <c r="B19" s="3" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="3:3">
       <c r="C22" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" spans="3:3">
       <c r="C23" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="3:3">
       <c r="C24" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" spans="3:3">
       <c r="C25" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="26" spans="3:3">
       <c r="C26" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="27" spans="3:3">
       <c r="C27" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="28" spans="3:3">
       <c r="C28" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" spans="3:3">
       <c r="C29" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="31" ht="21" spans="2:2">
       <c r="B31" s="3" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="33" spans="3:3">
       <c r="C33" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="34" spans="3:3">
       <c r="C34" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="35" spans="3:3">
       <c r="C35" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="36" spans="3:3">
       <c r="C36" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="38" spans="3:3">
       <c r="C38" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
     </row>
     <row r="39" spans="3:3">
       <c r="C39" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="3:3">
       <c r="C40" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="41" spans="3:3">
       <c r="C41" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -5750,7 +5762,7 @@
       <c r="H12" s="31"/>
       <c r="I12" s="30"/>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" ht="15.15" spans="1:9">
       <c r="A13" s="17"/>
       <c r="B13" s="32"/>
       <c r="C13" s="33" t="s">
@@ -5957,27 +5969,35 @@
       <c r="H23" s="51"/>
       <c r="I23" s="43"/>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" ht="28.8" spans="1:9">
       <c r="A24" s="17"/>
       <c r="B24" s="25"/>
       <c r="C24" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="D24" s="58"/>
-      <c r="E24" s="49"/>
+      <c r="D24" s="27" t="s">
+        <v>177</v>
+      </c>
+      <c r="E24" s="28" t="s">
+        <v>178</v>
+      </c>
       <c r="F24" s="50"/>
       <c r="G24" s="43"/>
       <c r="H24" s="51"/>
       <c r="I24" s="43"/>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" ht="15.15" spans="1:9">
       <c r="A25" s="17"/>
       <c r="B25" s="32"/>
       <c r="C25" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="D25" s="59"/>
-      <c r="E25" s="45"/>
+      <c r="D25" s="59" t="s">
+        <v>179</v>
+      </c>
+      <c r="E25" s="45" t="s">
+        <v>180</v>
+      </c>
       <c r="F25" s="55"/>
       <c r="G25" s="47"/>
       <c r="H25" s="56"/>
@@ -5985,10 +6005,10 @@
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="17" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C26" s="19" t="s">
         <v>110</v>
@@ -6026,7 +6046,7 @@
       <c r="H28" s="51"/>
       <c r="I28" s="43"/>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" ht="15.15" spans="1:9">
       <c r="A29" s="17"/>
       <c r="B29" s="32"/>
       <c r="C29" s="33" t="s">
@@ -6041,10 +6061,10 @@
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="17" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C30" s="19" t="s">
         <v>110</v>
@@ -6082,7 +6102,7 @@
       <c r="H32" s="51"/>
       <c r="I32" s="43"/>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" ht="15.15" spans="1:9">
       <c r="A33" s="17"/>
       <c r="B33" s="32"/>
       <c r="C33" s="33" t="s">
@@ -6097,10 +6117,10 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" s="17" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C34" s="19" t="s">
         <v>110</v>
@@ -6138,7 +6158,7 @@
       <c r="H36" s="51"/>
       <c r="I36" s="43"/>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" ht="15.15" spans="1:9">
       <c r="A37" s="17"/>
       <c r="B37" s="32"/>
       <c r="C37" s="33" t="s">
@@ -6153,10 +6173,10 @@
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="17" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B38" s="60" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C38" s="19" t="s">
         <v>110</v>
@@ -6188,7 +6208,7 @@
         <v>120</v>
       </c>
       <c r="D40" s="58" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="E40" s="49"/>
       <c r="F40" s="50"/>
@@ -6196,7 +6216,7 @@
       <c r="H40" s="51"/>
       <c r="I40" s="43"/>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" ht="15.15" spans="1:9">
       <c r="A41" s="17"/>
       <c r="B41" s="62"/>
       <c r="C41" s="33" t="s">
@@ -6211,10 +6231,10 @@
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="17" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B42" s="60" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C42" s="19" t="s">
         <v>110</v>
@@ -6252,7 +6272,7 @@
       <c r="H44" s="51"/>
       <c r="I44" s="43"/>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" ht="15.15" spans="1:9">
       <c r="A45" s="17"/>
       <c r="B45" s="62"/>
       <c r="C45" s="33" t="s">
@@ -6267,10 +6287,10 @@
     </row>
     <row r="46" spans="1:9">
       <c r="A46" s="17" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B46" s="60" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C46" s="19" t="s">
         <v>110</v>
@@ -6308,7 +6328,7 @@
       <c r="H48" s="51"/>
       <c r="I48" s="43"/>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" ht="15.15" spans="1:9">
       <c r="A49" s="17"/>
       <c r="B49" s="62"/>
       <c r="C49" s="33" t="s">
@@ -6380,25 +6400,25 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="6" spans="14:14">
       <c r="N6" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="14:14">
       <c r="N8" s="6" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9" spans="14:18">
       <c r="N9" s="7" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="R9" s="67" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -6425,7 +6445,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -6451,35 +6471,35 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="2:2">
       <c r="B20" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="2:2">
       <c r="B22" s="6" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23" customFormat="1" spans="2:6">
       <c r="B23" s="7" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="F23" s="68" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" spans="2:2">
       <c r="B24" s="7" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="25" spans="2:2">
       <c r="B25" s="7" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -6506,35 +6526,35 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" spans="3:3">
       <c r="C23" s="6" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="24" spans="3:3">
       <c r="C24" s="7" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="3:7">
       <c r="C25" s="7" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="G25" s="67" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="26" spans="3:3">
       <c r="C26" s="6" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -6561,30 +6581,30 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="14" spans="9:9">
       <c r="I14" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="9:9">
       <c r="I16" s="6" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="9:13">
       <c r="I17" s="7" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="M17" s="67" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" spans="9:9">
       <c r="I18" s="6" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>
@@ -6611,28 +6631,28 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" spans="13:13">
       <c r="M5" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" spans="13:17">
       <c r="M6" s="7" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="Q6" s="68" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="13:17">
       <c r="M7" s="7" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="Q7" s="68" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>